<commit_message>
feat(internacional): bucle de los dictámenes de 9.°–11.° y antecedente de 2.°–8.°
Serie inc9 del bucle (55 dictámenes nuevos): el refutador sostuvo 46 y
reabrió 9; la réplica cambió 8 por unanimidad del rol:
- a «solo especialización»: ciclo del nitrógeno, química verde, técnicas de
  estructura orgánica, potencial eléctrico y astronomía multionda;
- oleaje y Planck a «sin referente»; reflexión interna total a «alineado»
  (núcleo de HK S1–3, JP 中1 y ON SNC2D).
Diagramas de fases se mantiene (EE se suma al núcleo: 2 países).

El antecedente de 9.°–11.° suma el núcleo de 2.°–8.° de HK, SG, EE, KR, TW
y ON (consenso.ANTECEDENTE_2_8), ya extraído y etiquetado, sin Vertex:
8 clases automáticas cambian y 4 quedan inciertas (al panel, serie inc9b).

La vuelta 2 de una serie solo toma sus propios cambios. Dos errores más de
la malla: fibra óptica por dispersión (G10-FIS-U16-16.6) y taxismo por
cinesis (G03-CIE-U5-5.3).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/internacional/Contraste_quimica.xlsx
+++ b/internacional/Contraste_quimica.xlsx
@@ -626,6 +626,9 @@
       <c r="G2" t="n">
         <v>8.5</v>
       </c>
+      <c r="H2" t="n">
+        <v>7</v>
+      </c>
       <c r="I2" t="n">
         <v>9.5</v>
       </c>
@@ -945,6 +948,9 @@
       <c r="G6" t="n">
         <v>6</v>
       </c>
+      <c r="H6" t="n">
+        <v>7</v>
+      </c>
       <c r="I6" t="n">
         <v>8</v>
       </c>
@@ -1024,6 +1030,9 @@
       <c r="G7" t="n">
         <v>6</v>
       </c>
+      <c r="H7" t="n">
+        <v>7</v>
+      </c>
       <c r="I7" t="n">
         <v>2</v>
       </c>
@@ -1034,10 +1043,10 @@
         <v>9</v>
       </c>
       <c r="L7" t="n">
-        <v>9.5</v>
+        <v>7.5</v>
       </c>
       <c r="M7" t="n">
-        <v>7</v>
+        <v>4.5</v>
       </c>
       <c r="O7" t="n">
         <v>1</v>
@@ -1194,6 +1203,9 @@
       <c r="G9" t="n">
         <v>8.5</v>
       </c>
+      <c r="H9" t="n">
+        <v>7</v>
+      </c>
       <c r="I9" t="n">
         <v>8</v>
       </c>
@@ -1489,11 +1501,14 @@
       <c r="G13" t="n">
         <v>8.5</v>
       </c>
+      <c r="H13" t="n">
+        <v>7</v>
+      </c>
       <c r="J13" t="n">
         <v>9</v>
       </c>
       <c r="L13" t="n">
-        <v>9.5</v>
+        <v>7.5</v>
       </c>
       <c r="M13" t="n">
         <v>9.5</v>
@@ -2092,7 +2107,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Isomería estructural</t>
+          <t>Indicadores ácido-base</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -2101,41 +2116,56 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D21" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F21" t="n">
         <v>8</v>
       </c>
+      <c r="G21" t="n">
+        <v>6</v>
+      </c>
+      <c r="H21" t="n">
+        <v>7</v>
+      </c>
+      <c r="I21" t="n">
+        <v>5</v>
+      </c>
+      <c r="J21" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="K21" t="n">
+        <v>9</v>
+      </c>
       <c r="L21" t="n">
-        <v>11</v>
+        <v>7.5</v>
       </c>
       <c r="M21" t="n">
-        <v>7</v>
+        <v>2.5</v>
       </c>
       <c r="O21" t="n">
         <v>1</v>
       </c>
+      <c r="S21" t="n">
+        <v>1</v>
+      </c>
+      <c r="T21" t="n">
+        <v>1</v>
+      </c>
       <c r="U21" t="n">
         <v>1</v>
       </c>
       <c r="W21" t="n">
         <v>1</v>
       </c>
-      <c r="X21" t="n">
-        <v>1</v>
-      </c>
       <c r="Y21" t="n">
         <v>1</v>
       </c>
       <c r="Z21" t="n">
         <v>1</v>
       </c>
-      <c r="AA21" t="n">
-        <v>1</v>
-      </c>
       <c r="AC21" t="n">
         <v>1</v>
       </c>
@@ -2146,11 +2176,11 @@
         <v>1</v>
       </c>
       <c r="AF21" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="AG21" t="inlineStr">
         <is>
-          <t>sin_referente</t>
+          <t>alineado</t>
         </is>
       </c>
       <c r="AH21" t="inlineStr">
@@ -2162,7 +2192,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Leyes ponderales y volumétricas</t>
+          <t>Isomería estructural</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -2176,19 +2206,43 @@
       <c r="D22" t="n">
         <v>10</v>
       </c>
-      <c r="I22" t="n">
+      <c r="F22" t="n">
+        <v>8</v>
+      </c>
+      <c r="L22" t="n">
+        <v>11</v>
+      </c>
+      <c r="M22" t="n">
         <v>7</v>
       </c>
-      <c r="J22" t="n">
-        <v>7</v>
-      </c>
-      <c r="M22" t="n">
-        <v>9.5</v>
-      </c>
-      <c r="V22" t="n">
+      <c r="O22" t="n">
+        <v>1</v>
+      </c>
+      <c r="U22" t="n">
+        <v>1</v>
+      </c>
+      <c r="W22" t="n">
+        <v>1</v>
+      </c>
+      <c r="X22" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y22" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z22" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA22" t="n">
         <v>1</v>
       </c>
       <c r="AC22" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD22" t="n">
+        <v>1</v>
+      </c>
+      <c r="AE22" t="n">
         <v>1</v>
       </c>
       <c r="AF22" t="n">
@@ -2196,7 +2250,7 @@
       </c>
       <c r="AG22" t="inlineStr">
         <is>
-          <t>alineado</t>
+          <t>sin_referente</t>
         </is>
       </c>
       <c r="AH22" t="inlineStr">
@@ -2208,7 +2262,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Neutralización y reacciones de los ácidos</t>
+          <t>Leyes ponderales y volumétricas</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -2217,73 +2271,28 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D23" t="n">
-        <v>9</v>
-      </c>
-      <c r="F23" t="n">
-        <v>8</v>
-      </c>
-      <c r="G23" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="I23" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="J23" t="n">
-        <v>9</v>
-      </c>
-      <c r="K23" t="n">
-        <v>9</v>
-      </c>
-      <c r="L23" t="n">
+        <v>7</v>
+      </c>
+      <c r="M23" t="n">
         <v>9.5</v>
       </c>
-      <c r="M23" t="n">
-        <v>7</v>
-      </c>
-      <c r="O23" t="n">
-        <v>1</v>
-      </c>
-      <c r="P23" t="n">
-        <v>1</v>
-      </c>
-      <c r="R23" t="n">
-        <v>1</v>
-      </c>
-      <c r="S23" t="n">
-        <v>1</v>
-      </c>
-      <c r="T23" t="n">
-        <v>1</v>
-      </c>
-      <c r="U23" t="n">
-        <v>1</v>
-      </c>
-      <c r="W23" t="n">
-        <v>1</v>
-      </c>
-      <c r="Y23" t="n">
-        <v>1</v>
-      </c>
-      <c r="Z23" t="n">
-        <v>1</v>
-      </c>
-      <c r="AB23" t="n">
+      <c r="V23" t="n">
         <v>1</v>
       </c>
       <c r="AC23" t="n">
         <v>1</v>
       </c>
-      <c r="AD23" t="n">
-        <v>1</v>
-      </c>
-      <c r="AE23" t="n">
-        <v>1</v>
-      </c>
       <c r="AF23" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="AG23" t="inlineStr">
         <is>
@@ -2299,7 +2308,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Nomenclatura orgánica IUPAC</t>
+          <t>Neutralización y reacciones de los ácidos</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -2308,19 +2317,34 @@
         </is>
       </c>
       <c r="C24" t="n">
+        <v>9</v>
+      </c>
+      <c r="D24" t="n">
+        <v>9</v>
+      </c>
+      <c r="F24" t="n">
+        <v>8</v>
+      </c>
+      <c r="G24" t="n">
+        <v>6</v>
+      </c>
+      <c r="H24" t="n">
         <v>7</v>
       </c>
-      <c r="D24" t="n">
-        <v>11</v>
-      </c>
-      <c r="F24" t="n">
-        <v>10.5</v>
-      </c>
-      <c r="G24" t="n">
-        <v>8.5</v>
+      <c r="I24" t="n">
+        <v>8</v>
+      </c>
+      <c r="J24" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="K24" t="n">
+        <v>9</v>
       </c>
       <c r="L24" t="n">
-        <v>9.5</v>
+        <v>7.5</v>
+      </c>
+      <c r="M24" t="n">
+        <v>4.5</v>
       </c>
       <c r="O24" t="n">
         <v>1</v>
@@ -2328,15 +2352,21 @@
       <c r="P24" t="n">
         <v>1</v>
       </c>
+      <c r="R24" t="n">
+        <v>1</v>
+      </c>
+      <c r="S24" t="n">
+        <v>1</v>
+      </c>
+      <c r="T24" t="n">
+        <v>1</v>
+      </c>
       <c r="U24" t="n">
         <v>1</v>
       </c>
       <c r="W24" t="n">
         <v>1</v>
       </c>
-      <c r="X24" t="n">
-        <v>1</v>
-      </c>
       <c r="Y24" t="n">
         <v>1</v>
       </c>
@@ -2356,11 +2386,11 @@
         <v>1</v>
       </c>
       <c r="AF24" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="AG24" t="inlineStr">
         <is>
-          <t>retomado</t>
+          <t>alineado</t>
         </is>
       </c>
       <c r="AH24" t="inlineStr">
@@ -2372,7 +2402,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Oxidación y reducción</t>
+          <t>Nomenclatura orgánica IUPAC</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -2381,47 +2411,29 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="D25" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F25" t="n">
-        <v>8</v>
+        <v>10.5</v>
       </c>
       <c r="G25" t="n">
-        <v>6</v>
-      </c>
-      <c r="I25" t="n">
-        <v>7</v>
-      </c>
-      <c r="J25" t="n">
-        <v>9</v>
+        <v>8.5</v>
       </c>
       <c r="L25" t="n">
         <v>9.5</v>
       </c>
-      <c r="M25" t="n">
-        <v>7</v>
-      </c>
       <c r="O25" t="n">
         <v>1</v>
       </c>
       <c r="P25" t="n">
         <v>1</v>
       </c>
-      <c r="R25" t="n">
-        <v>1</v>
-      </c>
-      <c r="S25" t="n">
-        <v>1</v>
-      </c>
       <c r="U25" t="n">
         <v>1</v>
       </c>
-      <c r="V25" t="n">
-        <v>1</v>
-      </c>
       <c r="W25" t="n">
         <v>1</v>
       </c>
@@ -2432,9 +2444,6 @@
         <v>1</v>
       </c>
       <c r="Z25" t="n">
-        <v>1</v>
-      </c>
-      <c r="AA25" t="n">
         <v>1</v>
       </c>
       <c r="AB25" t="n">
@@ -2454,19 +2463,19 @@
       </c>
       <c r="AG25" t="inlineStr">
         <is>
+          <t>retomado</t>
+        </is>
+      </c>
+      <c r="AH25" t="inlineStr">
+        <is>
           <t>alineado</t>
-        </is>
-      </c>
-      <c r="AH25" t="inlineStr">
-        <is>
-          <t>tardio</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Polímeros y ambiente</t>
+          <t>Oxidación y reducción</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -2475,16 +2484,28 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D26" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F26" t="n">
         <v>8</v>
       </c>
+      <c r="G26" t="n">
+        <v>6</v>
+      </c>
+      <c r="H26" t="n">
+        <v>7</v>
+      </c>
+      <c r="I26" t="n">
+        <v>7</v>
+      </c>
+      <c r="J26" t="n">
+        <v>9</v>
+      </c>
       <c r="L26" t="n">
-        <v>9.5</v>
+        <v>7.5</v>
       </c>
       <c r="M26" t="n">
         <v>7</v>
@@ -2492,19 +2513,46 @@
       <c r="O26" t="n">
         <v>1</v>
       </c>
+      <c r="P26" t="n">
+        <v>1</v>
+      </c>
+      <c r="R26" t="n">
+        <v>1</v>
+      </c>
+      <c r="S26" t="n">
+        <v>1</v>
+      </c>
       <c r="U26" t="n">
         <v>1</v>
       </c>
+      <c r="V26" t="n">
+        <v>1</v>
+      </c>
       <c r="W26" t="n">
         <v>1</v>
       </c>
+      <c r="X26" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y26" t="n">
+        <v>1</v>
+      </c>
       <c r="Z26" t="n">
         <v>1</v>
       </c>
+      <c r="AA26" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB26" t="n">
+        <v>1</v>
+      </c>
       <c r="AC26" t="n">
         <v>1</v>
       </c>
       <c r="AD26" t="n">
+        <v>1</v>
+      </c>
+      <c r="AE26" t="n">
         <v>1</v>
       </c>
       <c r="AF26" t="n">
@@ -2512,19 +2560,19 @@
       </c>
       <c r="AG26" t="inlineStr">
         <is>
-          <t>sin_referente</t>
+          <t>alineado</t>
         </is>
       </c>
       <c r="AH26" t="inlineStr">
         <is>
-          <t>alineado</t>
+          <t>tardio</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Principio de Le Chatelier</t>
+          <t>Polímeros y ambiente</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -2533,19 +2581,19 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D27" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F27" t="n">
-        <v>10.5</v>
-      </c>
-      <c r="G27" t="n">
-        <v>8.5</v>
+        <v>8</v>
+      </c>
+      <c r="H27" t="n">
+        <v>7</v>
       </c>
       <c r="L27" t="n">
-        <v>11</v>
+        <v>9.5</v>
       </c>
       <c r="M27" t="n">
         <v>7</v>
@@ -2553,41 +2601,23 @@
       <c r="O27" t="n">
         <v>1</v>
       </c>
-      <c r="P27" t="n">
-        <v>1</v>
-      </c>
       <c r="U27" t="n">
         <v>1</v>
       </c>
       <c r="W27" t="n">
         <v>1</v>
       </c>
-      <c r="X27" t="n">
-        <v>1</v>
-      </c>
-      <c r="Y27" t="n">
-        <v>1</v>
-      </c>
       <c r="Z27" t="n">
         <v>1</v>
       </c>
-      <c r="AA27" t="n">
-        <v>1</v>
-      </c>
-      <c r="AB27" t="n">
-        <v>1</v>
-      </c>
       <c r="AC27" t="n">
         <v>1</v>
       </c>
       <c r="AD27" t="n">
         <v>1</v>
       </c>
-      <c r="AE27" t="n">
-        <v>1</v>
-      </c>
       <c r="AF27" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="AG27" t="inlineStr">
         <is>
@@ -2603,7 +2633,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Química de los carbohidratos</t>
+          <t>Principio de Le Chatelier</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -2612,35 +2642,32 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="D28" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F28" t="n">
         <v>10.5</v>
       </c>
-      <c r="I28" t="n">
-        <v>9.5</v>
+      <c r="G28" t="n">
+        <v>8.5</v>
       </c>
       <c r="L28" t="n">
-        <v>9.5</v>
+        <v>11</v>
       </c>
       <c r="M28" t="n">
-        <v>9.5</v>
+        <v>7</v>
       </c>
       <c r="O28" t="n">
         <v>1</v>
       </c>
-      <c r="R28" t="n">
+      <c r="P28" t="n">
         <v>1</v>
       </c>
       <c r="U28" t="n">
         <v>1</v>
       </c>
-      <c r="V28" t="n">
-        <v>1</v>
-      </c>
       <c r="W28" t="n">
         <v>1</v>
       </c>
@@ -2656,12 +2683,24 @@
       <c r="AA28" t="n">
         <v>1</v>
       </c>
+      <c r="AB28" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC28" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD28" t="n">
+        <v>1</v>
+      </c>
+      <c r="AE28" t="n">
+        <v>1</v>
+      </c>
       <c r="AF28" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="AG28" t="inlineStr">
         <is>
-          <t>retomado</t>
+          <t>alineado</t>
         </is>
       </c>
       <c r="AH28" t="inlineStr">
@@ -2673,7 +2712,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Química verde y economía atómica</t>
+          <t>Química de los carbohidratos</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -2682,16 +2721,16 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="D29" t="n">
-        <v>11</v>
-      </c>
-      <c r="G29" t="n">
-        <v>8.5</v>
-      </c>
-      <c r="K29" t="n">
-        <v>8</v>
+        <v>10</v>
+      </c>
+      <c r="F29" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="I29" t="n">
+        <v>9.5</v>
       </c>
       <c r="L29" t="n">
         <v>9.5</v>
@@ -2699,7 +2738,10 @@
       <c r="M29" t="n">
         <v>9.5</v>
       </c>
-      <c r="P29" t="n">
+      <c r="O29" t="n">
+        <v>1</v>
+      </c>
+      <c r="R29" t="n">
         <v>1</v>
       </c>
       <c r="U29" t="n">
@@ -2720,21 +2762,15 @@
       <c r="Z29" t="n">
         <v>1</v>
       </c>
-      <c r="AB29" t="n">
-        <v>1</v>
-      </c>
-      <c r="AC29" t="n">
-        <v>1</v>
-      </c>
-      <c r="AE29" t="n">
+      <c r="AA29" t="n">
         <v>1</v>
       </c>
       <c r="AF29" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="AG29" t="inlineStr">
         <is>
-          <t>sin_referente</t>
+          <t>retomado</t>
         </is>
       </c>
       <c r="AH29" t="inlineStr">
@@ -2818,11 +2854,14 @@
       <c r="G31" t="n">
         <v>8.5</v>
       </c>
+      <c r="H31" t="n">
+        <v>7</v>
+      </c>
       <c r="L31" t="n">
         <v>9.5</v>
       </c>
       <c r="M31" t="n">
-        <v>7</v>
+        <v>2.5</v>
       </c>
       <c r="N31" t="n">
         <v>1</v>
@@ -2903,6 +2942,9 @@
       <c r="G32" t="n">
         <v>8.5</v>
       </c>
+      <c r="H32" t="n">
+        <v>7</v>
+      </c>
       <c r="I32" t="n">
         <v>9.5</v>
       </c>
@@ -2944,7 +2986,7 @@
       </c>
       <c r="AG32" t="inlineStr">
         <is>
-          <t>sin_referente</t>
+          <t>alineado</t>
         </is>
       </c>
       <c r="AH32" t="inlineStr">
@@ -2979,6 +3021,9 @@
       <c r="G33" t="n">
         <v>6</v>
       </c>
+      <c r="H33" t="n">
+        <v>7</v>
+      </c>
       <c r="I33" t="n">
         <v>7</v>
       </c>
@@ -3229,10 +3274,10 @@
         <v>9.5</v>
       </c>
       <c r="J36" t="n">
-        <v>7</v>
+        <v>2.5</v>
       </c>
       <c r="M36" t="n">
-        <v>9.5</v>
+        <v>4.5</v>
       </c>
       <c r="O36" t="n">
         <v>1</v>
@@ -3463,12 +3508,12 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Técnicas para determinar estructuras orgánicas</t>
+          <t>Estructura y propiedades de los polímeros</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>no_aplica</t>
+          <t>incierto</t>
         </is>
       </c>
       <c r="C39" t="n">
@@ -3477,6 +3522,27 @@
       <c r="D39" t="n">
         <v>11</v>
       </c>
+      <c r="G39" t="n">
+        <v>6</v>
+      </c>
+      <c r="H39" t="n">
+        <v>7</v>
+      </c>
+      <c r="I39" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="L39" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="M39" t="n">
+        <v>7</v>
+      </c>
+      <c r="R39" t="n">
+        <v>1</v>
+      </c>
+      <c r="U39" t="n">
+        <v>1</v>
+      </c>
       <c r="W39" t="n">
         <v>1</v>
       </c>
@@ -3486,8 +3552,17 @@
       <c r="Z39" t="n">
         <v>1</v>
       </c>
-      <c r="AC39" t="n">
-        <v>1</v>
+      <c r="AA39" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD39" t="n">
+        <v>1</v>
+      </c>
+      <c r="AE39" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF39" t="n">
+        <v>11</v>
       </c>
       <c r="AG39" t="inlineStr">
         <is>
@@ -3496,7 +3571,7 @@
       </c>
       <c r="AH39" t="inlineStr">
         <is>
-          <t>no_aplica</t>
+          <t>tardio</t>
         </is>
       </c>
     </row>
@@ -3520,6 +3595,21 @@
       <c r="G40" t="n">
         <v>6</v>
       </c>
+      <c r="H40" t="n">
+        <v>2</v>
+      </c>
+      <c r="J40" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="K40" t="n">
+        <v>2</v>
+      </c>
+      <c r="L40" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="M40" t="n">
+        <v>2.5</v>
+      </c>
       <c r="AA40" t="n">
         <v>1</v>
       </c>
@@ -3557,6 +3647,9 @@
       <c r="F41" t="n">
         <v>8</v>
       </c>
+      <c r="H41" t="n">
+        <v>7</v>
+      </c>
       <c r="J41" t="n">
         <v>9</v>
       </c>
@@ -3694,20 +3787,23 @@
       <c r="G43" t="n">
         <v>6</v>
       </c>
+      <c r="H43" t="n">
+        <v>7</v>
+      </c>
       <c r="I43" t="n">
         <v>5</v>
       </c>
       <c r="J43" t="n">
-        <v>9</v>
+        <v>4.5</v>
       </c>
       <c r="K43" t="n">
         <v>9</v>
       </c>
       <c r="L43" t="n">
-        <v>9.5</v>
+        <v>7.5</v>
       </c>
       <c r="M43" t="n">
-        <v>7</v>
+        <v>2.5</v>
       </c>
       <c r="O43" t="n">
         <v>1</v>
@@ -3785,6 +3881,9 @@
       <c r="G44" t="n">
         <v>6</v>
       </c>
+      <c r="H44" t="n">
+        <v>7</v>
+      </c>
       <c r="I44" t="n">
         <v>8</v>
       </c>
@@ -3792,10 +3891,10 @@
         <v>7</v>
       </c>
       <c r="K44" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="L44" t="n">
-        <v>9.5</v>
+        <v>7.5</v>
       </c>
       <c r="M44" t="n">
         <v>7</v>
@@ -3882,17 +3981,23 @@
       <c r="G45" t="n">
         <v>2</v>
       </c>
+      <c r="H45" t="n">
+        <v>2</v>
+      </c>
       <c r="I45" t="n">
         <v>3</v>
       </c>
       <c r="J45" t="n">
-        <v>7</v>
+        <v>2.5</v>
+      </c>
+      <c r="K45" t="n">
+        <v>2</v>
       </c>
       <c r="L45" t="n">
-        <v>9.5</v>
+        <v>4</v>
       </c>
       <c r="M45" t="n">
-        <v>7</v>
+        <v>2.5</v>
       </c>
       <c r="O45" t="n">
         <v>1</v>
@@ -3973,20 +4078,23 @@
       <c r="G46" t="n">
         <v>2</v>
       </c>
+      <c r="H46" t="n">
+        <v>3</v>
+      </c>
       <c r="I46" t="n">
         <v>9.5</v>
       </c>
       <c r="J46" t="n">
-        <v>7</v>
+        <v>4.5</v>
       </c>
       <c r="K46" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="L46" t="n">
-        <v>9.5</v>
+        <v>7.5</v>
       </c>
       <c r="M46" t="n">
-        <v>7</v>
+        <v>4.5</v>
       </c>
       <c r="O46" t="n">
         <v>1</v>
@@ -4140,8 +4248,11 @@
       <c r="G48" t="n">
         <v>6</v>
       </c>
+      <c r="H48" t="n">
+        <v>3</v>
+      </c>
       <c r="K48" t="n">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="L48" t="n">
         <v>9.5</v>
@@ -4228,17 +4339,20 @@
       <c r="G49" t="n">
         <v>6</v>
       </c>
+      <c r="H49" t="n">
+        <v>3</v>
+      </c>
       <c r="I49" t="n">
         <v>5</v>
       </c>
       <c r="J49" t="n">
-        <v>9</v>
+        <v>4.5</v>
       </c>
       <c r="L49" t="n">
-        <v>9.5</v>
+        <v>7.5</v>
       </c>
       <c r="M49" t="n">
-        <v>7</v>
+        <v>2.5</v>
       </c>
       <c r="O49" t="n">
         <v>1</v>
@@ -4313,9 +4427,15 @@
       <c r="G50" t="n">
         <v>8.5</v>
       </c>
+      <c r="H50" t="n">
+        <v>2</v>
+      </c>
       <c r="I50" t="n">
         <v>5</v>
       </c>
+      <c r="J50" t="n">
+        <v>2.5</v>
+      </c>
       <c r="L50" t="n">
         <v>9.5</v>
       </c>
@@ -4375,13 +4495,22 @@
         <v>9</v>
       </c>
       <c r="F51" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="G51" t="n">
         <v>8.5</v>
       </c>
+      <c r="H51" t="n">
+        <v>2</v>
+      </c>
+      <c r="J51" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="K51" t="n">
+        <v>6</v>
+      </c>
       <c r="L51" t="n">
-        <v>9.5</v>
+        <v>7.5</v>
       </c>
       <c r="M51" t="n">
         <v>7</v>
@@ -4505,11 +4634,14 @@
       <c r="G53" t="n">
         <v>6</v>
       </c>
+      <c r="H53" t="n">
+        <v>7</v>
+      </c>
       <c r="I53" t="n">
         <v>9.5</v>
       </c>
       <c r="L53" t="n">
-        <v>9.5</v>
+        <v>7.5</v>
       </c>
       <c r="M53" t="n">
         <v>7</v>
@@ -4543,7 +4675,7 @@
       </c>
       <c r="AG53" t="inlineStr">
         <is>
-          <t>sin_referente</t>
+          <t>alineado</t>
         </is>
       </c>
       <c r="AH53" t="inlineStr">
@@ -4575,14 +4707,20 @@
       <c r="G54" t="n">
         <v>6</v>
       </c>
+      <c r="H54" t="n">
+        <v>7</v>
+      </c>
       <c r="I54" t="n">
         <v>2</v>
       </c>
       <c r="J54" t="n">
-        <v>7</v>
+        <v>4.5</v>
+      </c>
+      <c r="K54" t="n">
+        <v>6</v>
       </c>
       <c r="L54" t="n">
-        <v>9.5</v>
+        <v>7.5</v>
       </c>
       <c r="M54" t="n">
         <v>7</v>
@@ -4639,6 +4777,12 @@
       <c r="F55" t="n">
         <v>8</v>
       </c>
+      <c r="H55" t="n">
+        <v>7</v>
+      </c>
+      <c r="L55" t="n">
+        <v>7.5</v>
+      </c>
       <c r="M55" t="n">
         <v>7</v>
       </c>
@@ -4788,17 +4932,20 @@
       <c r="G57" t="n">
         <v>6</v>
       </c>
+      <c r="H57" t="n">
+        <v>7</v>
+      </c>
       <c r="I57" t="n">
         <v>7</v>
       </c>
       <c r="J57" t="n">
-        <v>7</v>
+        <v>4.5</v>
       </c>
       <c r="K57" t="n">
         <v>9</v>
       </c>
       <c r="L57" t="n">
-        <v>9.5</v>
+        <v>7.5</v>
       </c>
       <c r="M57" t="n">
         <v>7</v>
@@ -5198,6 +5345,9 @@
       <c r="G62" t="n">
         <v>8.5</v>
       </c>
+      <c r="H62" t="n">
+        <v>7</v>
+      </c>
       <c r="I62" t="n">
         <v>9.5</v>
       </c>
@@ -5283,17 +5433,23 @@
       <c r="G63" t="n">
         <v>6</v>
       </c>
+      <c r="H63" t="n">
+        <v>7</v>
+      </c>
       <c r="I63" t="n">
         <v>9.5</v>
       </c>
+      <c r="J63" t="n">
+        <v>4.5</v>
+      </c>
       <c r="K63" t="n">
         <v>9</v>
       </c>
       <c r="L63" t="n">
-        <v>9.5</v>
+        <v>7.5</v>
       </c>
       <c r="M63" t="n">
-        <v>7</v>
+        <v>4.5</v>
       </c>
       <c r="O63" t="n">
         <v>1</v>
@@ -5377,17 +5533,23 @@
       <c r="G64" t="n">
         <v>2</v>
       </c>
+      <c r="H64" t="n">
+        <v>2</v>
+      </c>
       <c r="I64" t="n">
         <v>3</v>
       </c>
       <c r="J64" t="n">
-        <v>7</v>
+        <v>2.5</v>
+      </c>
+      <c r="K64" t="n">
+        <v>2</v>
       </c>
       <c r="L64" t="n">
-        <v>9.5</v>
+        <v>4</v>
       </c>
       <c r="M64" t="n">
-        <v>7</v>
+        <v>2.5</v>
       </c>
       <c r="O64" t="n">
         <v>1</v>
@@ -5702,6 +5864,9 @@
       <c r="G68" t="n">
         <v>8.5</v>
       </c>
+      <c r="H68" t="n">
+        <v>7</v>
+      </c>
       <c r="I68" t="n">
         <v>9.5</v>
       </c>
@@ -5867,7 +6032,7 @@
         <v>9</v>
       </c>
       <c r="L70" t="n">
-        <v>9.5</v>
+        <v>7.5</v>
       </c>
       <c r="M70" t="n">
         <v>7</v>
@@ -5949,7 +6114,7 @@
         <v>9.5</v>
       </c>
       <c r="L71" t="n">
-        <v>9.5</v>
+        <v>7.5</v>
       </c>
       <c r="M71" t="n">
         <v>9.5</v>
@@ -6016,7 +6181,7 @@
         <v>8.5</v>
       </c>
       <c r="L72" t="n">
-        <v>9.5</v>
+        <v>7.5</v>
       </c>
       <c r="M72" t="n">
         <v>7</v>
@@ -6159,25 +6324,28 @@
         <v>2</v>
       </c>
       <c r="F74" t="n">
-        <v>8</v>
+        <v>2.5</v>
       </c>
       <c r="G74" t="n">
         <v>2</v>
       </c>
+      <c r="H74" t="n">
+        <v>2</v>
+      </c>
       <c r="I74" t="n">
         <v>6</v>
       </c>
       <c r="J74" t="n">
-        <v>7</v>
+        <v>2.5</v>
       </c>
       <c r="K74" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="L74" t="n">
-        <v>9.5</v>
+        <v>3</v>
       </c>
       <c r="M74" t="n">
-        <v>7</v>
+        <v>2.5</v>
       </c>
       <c r="O74" t="n">
         <v>1</v>
@@ -6249,17 +6417,20 @@
       <c r="G75" t="n">
         <v>8.5</v>
       </c>
+      <c r="H75" t="n">
+        <v>7</v>
+      </c>
       <c r="I75" t="n">
         <v>8</v>
       </c>
       <c r="J75" t="n">
-        <v>9</v>
+        <v>4.5</v>
       </c>
       <c r="K75" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="L75" t="n">
-        <v>9.5</v>
+        <v>7.5</v>
       </c>
       <c r="M75" t="n">
         <v>7</v>
@@ -6332,22 +6503,28 @@
         <v>6</v>
       </c>
       <c r="F76" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="G76" t="n">
         <v>6</v>
       </c>
+      <c r="H76" t="n">
+        <v>2</v>
+      </c>
       <c r="I76" t="n">
         <v>4</v>
       </c>
       <c r="J76" t="n">
-        <v>7</v>
+        <v>4.5</v>
+      </c>
+      <c r="K76" t="n">
+        <v>2</v>
       </c>
       <c r="L76" t="n">
-        <v>9.5</v>
+        <v>5</v>
       </c>
       <c r="M76" t="n">
-        <v>7</v>
+        <v>4.5</v>
       </c>
       <c r="O76" t="n">
         <v>1</v>
@@ -6416,6 +6593,9 @@
       <c r="G77" t="n">
         <v>6</v>
       </c>
+      <c r="H77" t="n">
+        <v>7</v>
+      </c>
       <c r="I77" t="n">
         <v>9.5</v>
       </c>
@@ -6423,10 +6603,10 @@
         <v>7</v>
       </c>
       <c r="K77" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="L77" t="n">
-        <v>9.5</v>
+        <v>7.5</v>
       </c>
       <c r="M77" t="n">
         <v>7</v>
@@ -6569,7 +6749,7 @@
         <v>8</v>
       </c>
       <c r="L79" t="n">
-        <v>9.5</v>
+        <v>7.5</v>
       </c>
       <c r="M79" t="n">
         <v>7</v>
@@ -6808,6 +6988,9 @@
       <c r="G82" t="n">
         <v>6</v>
       </c>
+      <c r="H82" t="n">
+        <v>7</v>
+      </c>
       <c r="I82" t="n">
         <v>7</v>
       </c>
@@ -6815,10 +6998,10 @@
         <v>7</v>
       </c>
       <c r="K82" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="L82" t="n">
-        <v>9.5</v>
+        <v>7.5</v>
       </c>
       <c r="M82" t="n">
         <v>7</v>
@@ -7003,6 +7186,9 @@
       <c r="F85" t="n">
         <v>10.5</v>
       </c>
+      <c r="H85" t="n">
+        <v>3</v>
+      </c>
       <c r="I85" t="n">
         <v>9.5</v>
       </c>
@@ -7016,7 +7202,7 @@
         <v>9.5</v>
       </c>
       <c r="M85" t="n">
-        <v>7</v>
+        <v>2.5</v>
       </c>
       <c r="O85" t="n">
         <v>1</v>
@@ -7085,6 +7271,9 @@
       <c r="I86" t="n">
         <v>9.5</v>
       </c>
+      <c r="K86" t="n">
+        <v>6</v>
+      </c>
       <c r="L86" t="n">
         <v>11</v>
       </c>
@@ -7164,6 +7353,12 @@
       <c r="G87" t="n">
         <v>3</v>
       </c>
+      <c r="H87" t="n">
+        <v>7</v>
+      </c>
+      <c r="K87" t="n">
+        <v>6</v>
+      </c>
       <c r="M87" t="n">
         <v>7</v>
       </c>
@@ -7219,6 +7414,9 @@
       <c r="G88" t="n">
         <v>6</v>
       </c>
+      <c r="K88" t="n">
+        <v>4</v>
+      </c>
       <c r="M88" t="n">
         <v>9.5</v>
       </c>
@@ -7327,22 +7525,28 @@
         <v>2</v>
       </c>
       <c r="F90" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="G90" t="n">
         <v>2</v>
       </c>
+      <c r="H90" t="n">
+        <v>2</v>
+      </c>
       <c r="I90" t="n">
         <v>9.5</v>
       </c>
       <c r="J90" t="n">
-        <v>7</v>
+        <v>2.5</v>
+      </c>
+      <c r="K90" t="n">
+        <v>2</v>
       </c>
       <c r="L90" t="n">
-        <v>9.5</v>
+        <v>3</v>
       </c>
       <c r="M90" t="n">
-        <v>7</v>
+        <v>2.5</v>
       </c>
       <c r="O90" t="n">
         <v>1</v>
@@ -7406,25 +7610,28 @@
         <v>9</v>
       </c>
       <c r="F91" t="n">
-        <v>8</v>
+        <v>2.5</v>
       </c>
       <c r="G91" t="n">
         <v>6</v>
       </c>
+      <c r="H91" t="n">
+        <v>2</v>
+      </c>
       <c r="I91" t="n">
         <v>6</v>
       </c>
       <c r="J91" t="n">
-        <v>7</v>
+        <v>2.5</v>
       </c>
       <c r="K91" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="L91" t="n">
-        <v>9.5</v>
+        <v>7.5</v>
       </c>
       <c r="M91" t="n">
-        <v>7</v>
+        <v>4.5</v>
       </c>
       <c r="O91" t="n">
         <v>1</v>
@@ -7599,15 +7806,24 @@
       <c r="D93" t="n">
         <v>9</v>
       </c>
+      <c r="F93" t="n">
+        <v>5</v>
+      </c>
       <c r="G93" t="n">
         <v>6</v>
       </c>
+      <c r="H93" t="n">
+        <v>7</v>
+      </c>
       <c r="I93" t="n">
         <v>3</v>
       </c>
       <c r="J93" t="n">
         <v>9</v>
       </c>
+      <c r="K93" t="n">
+        <v>2</v>
+      </c>
       <c r="L93" t="n">
         <v>11</v>
       </c>
@@ -7727,6 +7943,9 @@
       <c r="G95" t="n">
         <v>6</v>
       </c>
+      <c r="H95" t="n">
+        <v>7</v>
+      </c>
       <c r="I95" t="n">
         <v>9.5</v>
       </c>
@@ -7815,20 +8034,23 @@
       <c r="G96" t="n">
         <v>3</v>
       </c>
+      <c r="H96" t="n">
+        <v>5</v>
+      </c>
       <c r="I96" t="n">
         <v>5</v>
       </c>
       <c r="J96" t="n">
-        <v>7</v>
+        <v>4.5</v>
       </c>
       <c r="K96" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="L96" t="n">
-        <v>9.5</v>
+        <v>7.5</v>
       </c>
       <c r="M96" t="n">
-        <v>7</v>
+        <v>4.5</v>
       </c>
       <c r="O96" t="n">
         <v>1</v>
@@ -7962,22 +8184,28 @@
         <v>6</v>
       </c>
       <c r="F98" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="G98" t="n">
         <v>3</v>
       </c>
+      <c r="H98" t="n">
+        <v>2</v>
+      </c>
       <c r="I98" t="n">
         <v>4</v>
       </c>
       <c r="J98" t="n">
-        <v>7</v>
+        <v>4.5</v>
+      </c>
+      <c r="K98" t="n">
+        <v>6</v>
       </c>
       <c r="L98" t="n">
-        <v>9.5</v>
+        <v>7.5</v>
       </c>
       <c r="M98" t="n">
-        <v>7</v>
+        <v>2.5</v>
       </c>
       <c r="O98" t="n">
         <v>1</v>
@@ -8107,17 +8335,23 @@
       <c r="G100" t="n">
         <v>3</v>
       </c>
+      <c r="H100" t="n">
+        <v>2</v>
+      </c>
       <c r="I100" t="n">
         <v>4</v>
       </c>
       <c r="J100" t="n">
-        <v>7</v>
+        <v>4.5</v>
+      </c>
+      <c r="K100" t="n">
+        <v>6</v>
       </c>
       <c r="L100" t="n">
-        <v>9.5</v>
+        <v>7.5</v>
       </c>
       <c r="M100" t="n">
-        <v>9.5</v>
+        <v>2.5</v>
       </c>
       <c r="O100" t="n">
         <v>1</v>
@@ -8195,6 +8429,9 @@
       <c r="G101" t="n">
         <v>6</v>
       </c>
+      <c r="H101" t="n">
+        <v>7</v>
+      </c>
       <c r="I101" t="n">
         <v>7</v>
       </c>
@@ -8202,13 +8439,13 @@
         <v>7</v>
       </c>
       <c r="K101" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="L101" t="n">
-        <v>9.5</v>
+        <v>7.5</v>
       </c>
       <c r="M101" t="n">
-        <v>7</v>
+        <v>2.5</v>
       </c>
       <c r="O101" t="n">
         <v>1</v>
@@ -8286,6 +8523,9 @@
       <c r="G102" t="n">
         <v>6</v>
       </c>
+      <c r="H102" t="n">
+        <v>3</v>
+      </c>
       <c r="I102" t="n">
         <v>9.5</v>
       </c>
@@ -8296,7 +8536,7 @@
         <v>8</v>
       </c>
       <c r="L102" t="n">
-        <v>9.5</v>
+        <v>7.5</v>
       </c>
       <c r="M102" t="n">
         <v>7</v>
@@ -8386,6 +8626,9 @@
       <c r="G103" t="n">
         <v>8.5</v>
       </c>
+      <c r="H103" t="n">
+        <v>7</v>
+      </c>
       <c r="I103" t="n">
         <v>9.5</v>
       </c>
@@ -8483,6 +8726,9 @@
       <c r="G104" t="n">
         <v>6</v>
       </c>
+      <c r="H104" t="n">
+        <v>7</v>
+      </c>
       <c r="I104" t="n">
         <v>7</v>
       </c>
@@ -8490,7 +8736,7 @@
         <v>9</v>
       </c>
       <c r="L104" t="n">
-        <v>9.5</v>
+        <v>7.5</v>
       </c>
       <c r="N104" t="n">
         <v>1</v>
@@ -8554,11 +8800,20 @@
         <v>10</v>
       </c>
       <c r="F105" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="G105" t="n">
         <v>8.5</v>
       </c>
+      <c r="H105" t="n">
+        <v>2</v>
+      </c>
+      <c r="K105" t="n">
+        <v>2</v>
+      </c>
+      <c r="L105" t="n">
+        <v>5</v>
+      </c>
       <c r="M105" t="n">
         <v>7</v>
       </c>
@@ -8697,6 +8952,9 @@
       <c r="G108" t="n">
         <v>8.5</v>
       </c>
+      <c r="L108" t="n">
+        <v>7.5</v>
+      </c>
       <c r="AC108" t="n">
         <v>1</v>
       </c>
@@ -8772,7 +9030,7 @@
         <v>10</v>
       </c>
       <c r="J110" t="n">
-        <v>7</v>
+        <v>2.5</v>
       </c>
       <c r="M110" t="n">
         <v>9.5</v>
@@ -8957,6 +9215,9 @@
       <c r="J113" t="n">
         <v>7</v>
       </c>
+      <c r="L113" t="n">
+        <v>7.5</v>
+      </c>
       <c r="AA113" t="n">
         <v>1</v>
       </c>
@@ -8982,7 +9243,7 @@
       </c>
       <c r="AH113" t="inlineStr">
         <is>
-          <t>solo_especializacion</t>
+          <t>sin_referente</t>
         </is>
       </c>
     </row>
@@ -9352,6 +9613,9 @@
       <c r="D121" t="n">
         <v>10</v>
       </c>
+      <c r="H121" t="n">
+        <v>7</v>
+      </c>
       <c r="I121" t="n">
         <v>9.5</v>
       </c>
@@ -9393,7 +9657,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>Estereoquímica y quiralidad</t>
+          <t>Técnicas para determinar estructuras orgánicas</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
@@ -9402,21 +9666,12 @@
         </is>
       </c>
       <c r="C122" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D122" t="n">
-        <v>10</v>
-      </c>
-      <c r="L122" t="n">
         <v>11</v>
       </c>
-      <c r="M122" t="n">
-        <v>7</v>
-      </c>
-      <c r="U122" t="n">
-        <v>1</v>
-      </c>
-      <c r="X122" t="n">
+      <c r="W122" t="n">
         <v>1</v>
       </c>
       <c r="Y122" t="n">
@@ -9425,21 +9680,9 @@
       <c r="Z122" t="n">
         <v>1</v>
       </c>
-      <c r="AA122" t="n">
-        <v>1</v>
-      </c>
       <c r="AC122" t="n">
         <v>1</v>
       </c>
-      <c r="AD122" t="n">
-        <v>1</v>
-      </c>
-      <c r="AE122" t="n">
-        <v>1</v>
-      </c>
-      <c r="AF122" t="n">
-        <v>11</v>
-      </c>
       <c r="AG122" t="inlineStr">
         <is>
           <t>solo_especializacion</t>
@@ -9447,14 +9690,14 @@
       </c>
       <c r="AH122" t="inlineStr">
         <is>
-          <t>solo_especializacion</t>
+          <t>no_aplica</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>Estructura y propiedades de los polímeros</t>
+          <t>Estereoquímica y quiralidad</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
@@ -9463,30 +9706,21 @@
         </is>
       </c>
       <c r="C123" t="n">
+        <v>10</v>
+      </c>
+      <c r="D123" t="n">
+        <v>10</v>
+      </c>
+      <c r="L123" t="n">
         <v>11</v>
-      </c>
-      <c r="D123" t="n">
-        <v>11</v>
-      </c>
-      <c r="G123" t="n">
-        <v>6</v>
-      </c>
-      <c r="I123" t="n">
-        <v>9.5</v>
-      </c>
-      <c r="L123" t="n">
-        <v>9.5</v>
       </c>
       <c r="M123" t="n">
         <v>7</v>
       </c>
-      <c r="R123" t="n">
-        <v>1</v>
-      </c>
       <c r="U123" t="n">
         <v>1</v>
       </c>
-      <c r="W123" t="n">
+      <c r="X123" t="n">
         <v>1</v>
       </c>
       <c r="Y123" t="n">
@@ -9496,6 +9730,9 @@
         <v>1</v>
       </c>
       <c r="AA123" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC123" t="n">
         <v>1</v>
       </c>
       <c r="AD123" t="n">
@@ -9686,7 +9923,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>Indicadores ácido-base</t>
+          <t>Ley de Hess y entalpías de formación</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
@@ -9695,53 +9932,47 @@
         </is>
       </c>
       <c r="C127" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D127" t="n">
-        <v>9</v>
-      </c>
-      <c r="F127" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="G127" t="n">
-        <v>6</v>
-      </c>
-      <c r="I127" t="n">
-        <v>5</v>
-      </c>
-      <c r="J127" t="n">
-        <v>9</v>
-      </c>
-      <c r="K127" t="n">
-        <v>9</v>
+        <v>8.5</v>
       </c>
       <c r="L127" t="n">
+        <v>11</v>
+      </c>
+      <c r="M127" t="n">
         <v>9.5</v>
       </c>
-      <c r="M127" t="n">
-        <v>7</v>
-      </c>
-      <c r="O127" t="n">
-        <v>1</v>
-      </c>
-      <c r="S127" t="n">
-        <v>1</v>
-      </c>
-      <c r="T127" t="n">
+      <c r="P127" t="n">
         <v>1</v>
       </c>
       <c r="U127" t="n">
         <v>1</v>
       </c>
+      <c r="V127" t="n">
+        <v>1</v>
+      </c>
       <c r="W127" t="n">
         <v>1</v>
       </c>
+      <c r="X127" t="n">
+        <v>1</v>
+      </c>
       <c r="Y127" t="n">
         <v>1</v>
       </c>
       <c r="Z127" t="n">
         <v>1</v>
       </c>
+      <c r="AA127" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB127" t="n">
+        <v>1</v>
+      </c>
       <c r="AC127" t="n">
         <v>1</v>
       </c>
@@ -9752,7 +9983,7 @@
         <v>1</v>
       </c>
       <c r="AF127" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="AG127" t="inlineStr">
         <is>
@@ -9768,7 +9999,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>Ley de Hess y entalpías de formación</t>
+          <t>Ley de velocidad, orden de reacción y ecuación de Arrhenius</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -9777,32 +10008,17 @@
         </is>
       </c>
       <c r="C128" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D128" t="n">
-        <v>10</v>
-      </c>
-      <c r="G128" t="n">
-        <v>8.5</v>
+        <v>9</v>
       </c>
       <c r="L128" t="n">
         <v>11</v>
       </c>
-      <c r="M128" t="n">
-        <v>9.5</v>
-      </c>
-      <c r="P128" t="n">
-        <v>1</v>
-      </c>
       <c r="U128" t="n">
         <v>1</v>
       </c>
-      <c r="V128" t="n">
-        <v>1</v>
-      </c>
-      <c r="W128" t="n">
-        <v>1</v>
-      </c>
       <c r="X128" t="n">
         <v>1</v>
       </c>
@@ -9810,9 +10026,6 @@
         <v>1</v>
       </c>
       <c r="Z128" t="n">
-        <v>1</v>
-      </c>
-      <c r="AA128" t="n">
         <v>1</v>
       </c>
       <c r="AB128" t="n">
@@ -9844,7 +10057,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>Ley de velocidad, orden de reacción y ecuación de Arrhenius</t>
+          <t>Mecanismos de reacción</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -9853,16 +10066,10 @@
         </is>
       </c>
       <c r="C129" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D129" t="n">
-        <v>9</v>
-      </c>
-      <c r="L129" t="n">
-        <v>11</v>
-      </c>
-      <c r="U129" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="X129" t="n">
         <v>1</v>
@@ -9873,16 +10080,10 @@
       <c r="Z129" t="n">
         <v>1</v>
       </c>
-      <c r="AB129" t="n">
-        <v>1</v>
-      </c>
       <c r="AC129" t="n">
         <v>1</v>
       </c>
       <c r="AD129" t="n">
-        <v>1</v>
-      </c>
-      <c r="AE129" t="n">
         <v>1</v>
       </c>
       <c r="AF129" t="n">
@@ -9902,7 +10103,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>Mecanismos de reacción</t>
+          <t>Nanomateriales y manufactura molecular</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
@@ -9911,12 +10112,15 @@
         </is>
       </c>
       <c r="C130" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D130" t="n">
-        <v>10</v>
-      </c>
-      <c r="X130" t="n">
+        <v>11</v>
+      </c>
+      <c r="G130" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="W130" t="n">
         <v>1</v>
       </c>
       <c r="Y130" t="n">
@@ -9925,14 +10129,11 @@
       <c r="Z130" t="n">
         <v>1</v>
       </c>
-      <c r="AC130" t="n">
-        <v>1</v>
-      </c>
-      <c r="AD130" t="n">
+      <c r="AE130" t="n">
         <v>1</v>
       </c>
       <c r="AF130" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="AG130" t="inlineStr">
         <is>
@@ -9948,7 +10149,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>Nanomateriales y manufactura molecular</t>
+          <t>Polimerización por adición y por condensación</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
@@ -9962,8 +10163,17 @@
       <c r="D131" t="n">
         <v>11</v>
       </c>
-      <c r="G131" t="n">
-        <v>8.5</v>
+      <c r="F131" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="L131" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="O131" t="n">
+        <v>1</v>
+      </c>
+      <c r="U131" t="n">
+        <v>1</v>
       </c>
       <c r="W131" t="n">
         <v>1</v>
@@ -9972,6 +10182,18 @@
         <v>1</v>
       </c>
       <c r="Z131" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA131" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB131" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC131" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD131" t="n">
         <v>1</v>
       </c>
       <c r="AE131" t="n">
@@ -9994,7 +10216,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>Polimerización por adición y por condensación</t>
+          <t>Potenciales estándar de electrodo y de celda</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -10003,33 +10225,39 @@
         </is>
       </c>
       <c r="C132" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D132" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F132" t="n">
-        <v>10.5</v>
-      </c>
-      <c r="L132" t="n">
+        <v>8</v>
+      </c>
+      <c r="G132" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="I132" t="n">
         <v>9.5</v>
       </c>
       <c r="O132" t="n">
         <v>1</v>
       </c>
-      <c r="U132" t="n">
+      <c r="P132" t="n">
+        <v>1</v>
+      </c>
+      <c r="R132" t="n">
         <v>1</v>
       </c>
       <c r="W132" t="n">
         <v>1</v>
       </c>
+      <c r="X132" t="n">
+        <v>1</v>
+      </c>
       <c r="Y132" t="n">
         <v>1</v>
       </c>
       <c r="Z132" t="n">
-        <v>1</v>
-      </c>
-      <c r="AA132" t="n">
         <v>1</v>
       </c>
       <c r="AB132" t="n">
@@ -10061,7 +10289,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>Potenciales estándar de electrodo y de celda</t>
+          <t>Producto de solubilidad (Kps)</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -10075,37 +10303,7 @@
       <c r="D133" t="n">
         <v>10</v>
       </c>
-      <c r="F133" t="n">
-        <v>8</v>
-      </c>
-      <c r="G133" t="n">
-        <v>8.5</v>
-      </c>
-      <c r="I133" t="n">
-        <v>9.5</v>
-      </c>
-      <c r="O133" t="n">
-        <v>1</v>
-      </c>
-      <c r="P133" t="n">
-        <v>1</v>
-      </c>
-      <c r="R133" t="n">
-        <v>1</v>
-      </c>
-      <c r="W133" t="n">
-        <v>1</v>
-      </c>
       <c r="X133" t="n">
-        <v>1</v>
-      </c>
-      <c r="Y133" t="n">
-        <v>1</v>
-      </c>
-      <c r="Z133" t="n">
-        <v>1</v>
-      </c>
-      <c r="AB133" t="n">
         <v>1</v>
       </c>
       <c r="AC133" t="n">
@@ -10134,7 +10332,7 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>Producto de solubilidad (Kps)</t>
+          <t>Química de los ácidos nucleicos</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
@@ -10148,20 +10346,20 @@
       <c r="D134" t="n">
         <v>10</v>
       </c>
-      <c r="X134" t="n">
-        <v>1</v>
-      </c>
-      <c r="AC134" t="n">
-        <v>1</v>
-      </c>
-      <c r="AD134" t="n">
-        <v>1</v>
-      </c>
-      <c r="AE134" t="n">
+      <c r="Y134" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z134" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA134" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB134" t="n">
         <v>1</v>
       </c>
       <c r="AF134" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="AG134" t="inlineStr">
         <is>
@@ -10177,7 +10375,7 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>Química de los ácidos nucleicos</t>
+          <t>Química verde y economía atómica</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
@@ -10186,10 +10384,40 @@
         </is>
       </c>
       <c r="C135" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D135" t="n">
-        <v>10</v>
+        <v>11</v>
+      </c>
+      <c r="G135" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="H135" t="n">
+        <v>7</v>
+      </c>
+      <c r="K135" t="n">
+        <v>4</v>
+      </c>
+      <c r="L135" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="M135" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="P135" t="n">
+        <v>1</v>
+      </c>
+      <c r="U135" t="n">
+        <v>1</v>
+      </c>
+      <c r="V135" t="n">
+        <v>1</v>
+      </c>
+      <c r="W135" t="n">
+        <v>1</v>
+      </c>
+      <c r="X135" t="n">
+        <v>1</v>
       </c>
       <c r="Y135" t="n">
         <v>1</v>
@@ -10197,23 +10425,26 @@
       <c r="Z135" t="n">
         <v>1</v>
       </c>
-      <c r="AA135" t="n">
-        <v>1</v>
-      </c>
       <c r="AB135" t="n">
         <v>1</v>
       </c>
+      <c r="AC135" t="n">
+        <v>1</v>
+      </c>
+      <c r="AE135" t="n">
+        <v>1</v>
+      </c>
       <c r="AF135" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="AG135" t="inlineStr">
         <is>
-          <t>solo_especializacion</t>
+          <t>alineado</t>
         </is>
       </c>
       <c r="AH135" t="inlineStr">
         <is>
-          <t>solo_especializacion</t>
+          <t>tardio</t>
         </is>
       </c>
     </row>

</xml_diff>